<commit_message>
:art: Update public demo for v0.4.59
</commit_message>
<xml_diff>
--- a/fh6-livery-organizer-demo.xlsx
+++ b/fh6-livery-organizer-demo.xlsx
@@ -1647,29 +1647,29 @@
   <dimension ref="A1:W51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="34" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="24" customWidth="1"/>
-    <col min="7" max="7" width="9" customWidth="1"/>
-    <col min="8" max="8" width="24" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="26" customWidth="1"/>
-    <col min="12" max="12" width="40" customWidth="1"/>
-    <col min="13" max="13" width="20" customWidth="1"/>
-    <col min="14" max="14" width="22" customWidth="1"/>
-    <col min="15" max="15" width="36" customWidth="1"/>
-    <col min="16" max="16" width="12" customWidth="1"/>
-    <col min="17" max="17" width="12" customWidth="1"/>
-    <col min="18" max="18" width="20" customWidth="1"/>
-    <col min="19" max="19" width="30" customWidth="1"/>
-    <col min="20" max="20" width="24" customWidth="1"/>
-    <col min="21" max="21" width="32" customWidth="1"/>
-    <col min="22" max="22" width="48" customWidth="1"/>
-    <col min="23" max="23" width="40" customWidth="1"/>
+    <col min="1" max="1" width="24.0" customWidth="1"/>
+    <col min="2" max="2" width="12.0" customWidth="1"/>
+    <col min="3" max="3" width="10.0" customWidth="1"/>
+    <col min="4" max="4" width="34.0" customWidth="1"/>
+    <col min="5" max="5" width="18.0" customWidth="1"/>
+    <col min="6" max="6" width="24.0" customWidth="1"/>
+    <col min="7" max="7" width="9.0" customWidth="1"/>
+    <col min="8" max="8" width="24.0" customWidth="1"/>
+    <col min="9" max="9" width="20.0" customWidth="1"/>
+    <col min="10" max="10" width="12.0" customWidth="1"/>
+    <col min="11" max="11" width="26.0" customWidth="1"/>
+    <col min="12" max="12" width="40.0" customWidth="1"/>
+    <col min="13" max="13" width="20.0" customWidth="1"/>
+    <col min="14" max="14" width="22.0" customWidth="1"/>
+    <col min="15" max="15" width="36.0" customWidth="1"/>
+    <col min="16" max="16" width="12.0" customWidth="1"/>
+    <col min="17" max="17" width="12.0" customWidth="1"/>
+    <col min="18" max="18" width="20.0" customWidth="1"/>
+    <col min="19" max="19" width="30.0" customWidth="1"/>
+    <col min="20" max="20" width="24.0" customWidth="1"/>
+    <col min="21" max="21" width="32.0" customWidth="1"/>
+    <col min="22" max="22" width="48.0" customWidth="1"/>
+    <col min="23" max="23" width="40.0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1801,38 +1801,38 @@
         </is>
       </c>
       <c r="C2" s="3">
-        <v>261</v>
+        <v>422</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1995 Porsche 911 GT2</t>
+          <t xml:space="preserve">2002 Acura RSX Type S</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Porsche</t>
+          <t xml:space="preserve">Acura</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">911 GT2</t>
+          <t xml:space="preserve">RSX Type S</t>
         </is>
       </c>
       <c r="G2" s="3">
-        <v>1995</v>
+        <v>2002</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_911gt2_95</t>
+          <t xml:space="preserve">ACU_RSXTypeS_02</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 17</t>
+          <t xml:space="preserve">Demo Creator 19</t>
         </is>
       </c>
       <c r="J2" s="3">
-        <v>10373</v>
+        <v>5349</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -1876,12 +1876,12 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_0261_001</t>
+          <t xml:space="preserve">DemoLivery_0422_001</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">b4c89edf496cd98a70837b0e</t>
+          <t xml:space="preserve">e779bec68dacd2f7f649e493</t>
         </is>
       </c>
       <c r="U2" s="2" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_0261_001</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_0422_001</t>
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr">
@@ -1912,38 +1912,38 @@
         </is>
       </c>
       <c r="C3" s="3">
-        <v>422</v>
+        <v>433</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2002 Acura RSX Type S</t>
+          <t xml:space="preserve">2005 TVR Sagaris</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Acura</t>
+          <t xml:space="preserve">TVR</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RSX Type S</t>
+          <t xml:space="preserve">Sagaris</t>
         </is>
       </c>
       <c r="G3" s="3">
-        <v>2002</v>
+        <v>2005</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACU_RSXTypeS_02</t>
+          <t xml:space="preserve">TVR_Sagaris_05</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 25</t>
+          <t xml:space="preserve">Demo Creator 29</t>
         </is>
       </c>
       <c r="J3" s="3">
-        <v>10546</v>
+        <v>1426</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -1987,12 +1987,12 @@
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_0422_002</t>
+          <t xml:space="preserve">DemoLivery_0433_002</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8f989cae49306414880e8059</t>
+          <t xml:space="preserve">d253434b6fa446c3d7c12706</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_0422_002</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_0433_002</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
@@ -2023,38 +2023,38 @@
         </is>
       </c>
       <c r="C4" s="3">
-        <v>433</v>
+        <v>1045</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2005 TVR Sagaris</t>
+          <t xml:space="preserve">1987 Pontiac Firebird Trans Am GTA</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TVR</t>
+          <t xml:space="preserve">Pontiac</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sagaris</t>
+          <t xml:space="preserve">Firebird Trans Am GTA</t>
         </is>
       </c>
       <c r="G4" s="3">
-        <v>2005</v>
+        <v>1987</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TVR_Sagaris_05</t>
+          <t xml:space="preserve">PON_TransAmGTA_87</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 29</t>
+          <t xml:space="preserve">Demo Creator 23</t>
         </is>
       </c>
       <c r="J4" s="3">
-        <v>1539</v>
+        <v>293</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -2098,12 +2098,12 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_0433_003</t>
+          <t xml:space="preserve">DemoLivery_1045_003</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0d406b0cdaabf616b98776dc</t>
+          <t xml:space="preserve">efc8f432903d355f23d3e464</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_0433_003</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1045_003</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
@@ -2134,38 +2134,38 @@
         </is>
       </c>
       <c r="C5" s="3">
-        <v>1045</v>
+        <v>1124</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1987 Pontiac Firebird Trans Am GTA</t>
+          <t xml:space="preserve">1980 Abarth Fiat 131</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pontiac</t>
+          <t xml:space="preserve">Abarth</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Firebird Trans Am GTA</t>
+          <t xml:space="preserve">Fiat 131</t>
         </is>
       </c>
       <c r="G5" s="3">
-        <v>1987</v>
+        <v>1980</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PON_TransAmGTA_87</t>
+          <t xml:space="preserve">FIA_131AbarthStradale_80</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 23</t>
+          <t xml:space="preserve">Demo Creator 15</t>
         </is>
       </c>
       <c r="J5" s="3">
-        <v>364</v>
+        <v>5796</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
@@ -2209,12 +2209,12 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_1045_004</t>
+          <t xml:space="preserve">DemoLivery_1124_004</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">c4be68271ca9586015ca6e85</t>
+          <t xml:space="preserve">e466dd5765184bfee303014d</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1045_004</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1124_004</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr">
@@ -2245,38 +2245,38 @@
         </is>
       </c>
       <c r="C6" s="3">
-        <v>1124</v>
+        <v>1130</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1980 Abarth Fiat 131</t>
+          <t xml:space="preserve">2011 McLaren 12C Coupé</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abarth</t>
+          <t xml:space="preserve">McLaren</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fiat 131</t>
+          <t xml:space="preserve">12C Coupé</t>
         </is>
       </c>
       <c r="G6" s="3">
-        <v>1980</v>
+        <v>2011</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FIA_131AbarthStradale_80</t>
+          <t xml:space="preserve">MCL_MP412C_11</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 16</t>
+          <t xml:space="preserve">Demo Creator 37</t>
         </is>
       </c>
       <c r="J6" s="3">
-        <v>5945</v>
+        <v>11065</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -2320,12 +2320,12 @@
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_1124_005</t>
+          <t xml:space="preserve">DemoLivery_1130_005</t>
         </is>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ace710ef09e0eb7c22b39017</t>
+          <t xml:space="preserve">7902fafe68f3da51050fc790</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1124_005</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1130_005</t>
         </is>
       </c>
       <c r="W6" s="2" t="inlineStr">
@@ -2356,38 +2356,38 @@
         </is>
       </c>
       <c r="C7" s="3">
-        <v>1130</v>
+        <v>1270</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2011 McLaren 12C Coupé</t>
+          <t xml:space="preserve">1982 DeLorean DMC-12</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">McLaren</t>
+          <t xml:space="preserve">DeLorean</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">12C Coupé</t>
+          <t xml:space="preserve">DMC-12</t>
         </is>
       </c>
       <c r="G7" s="3">
-        <v>2011</v>
+        <v>1982</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCL_MP412C_11</t>
+          <t xml:space="preserve">DEL_DMC12_82</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 37</t>
+          <t xml:space="preserve">Demo Creator 25</t>
         </is>
       </c>
       <c r="J7" s="3">
-        <v>11238</v>
+        <v>6094</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
@@ -2431,12 +2431,12 @@
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_1130_006</t>
+          <t xml:space="preserve">DemoLivery_1270_006</t>
         </is>
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">381e3f4779caff9c99969816</t>
+          <t xml:space="preserve">47cb49916fb141df51576857</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1130_006</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1270_006</t>
         </is>
       </c>
       <c r="W7" s="2" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 14</t>
+          <t xml:space="preserve">Demo Creator 13</t>
         </is>
       </c>
       <c r="J9" s="3">
@@ -2658,7 +2658,7 @@
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1124bdfee369eccc325b6217</t>
+          <t xml:space="preserve">1435f6e3896f96fffb44b7e0</t>
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 18</t>
+          <t xml:space="preserve">Demo Creator 16</t>
         </is>
       </c>
       <c r="J11" s="3">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">c0ec333180726a66c252edc2</t>
+          <t xml:space="preserve">295ba194f516f7b88564a168</t>
         </is>
       </c>
       <c r="U11" s="2" t="inlineStr">
@@ -2938,7 +2938,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 22</t>
+          <t xml:space="preserve">Demo Creator 20</t>
         </is>
       </c>
       <c r="J12" s="3">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">53b89fd59ff5584956a10421</t>
+          <t xml:space="preserve">359893763b8db363960bbb34</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
@@ -3271,7 +3271,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 32</t>
+          <t xml:space="preserve">Demo Creator 31</t>
         </is>
       </c>
       <c r="J15" s="3">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="T15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4bf4cd189bd4b3fb3b5d8b7d</t>
+          <t xml:space="preserve">fbc466f459e9bd8f085b409a</t>
         </is>
       </c>
       <c r="U15" s="2" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 20</t>
+          <t xml:space="preserve">Demo Creator 18</t>
         </is>
       </c>
       <c r="J18" s="3">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">25c4da96ec7aa398cbefbefc</t>
+          <t xml:space="preserve">5663cb081a5208f00fc0e669</t>
         </is>
       </c>
       <c r="U18" s="2" t="inlineStr">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 19</t>
+          <t xml:space="preserve">Demo Creator 17</t>
         </is>
       </c>
       <c r="J20" s="3">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="T20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">68fde6f89f149ab63681ce1c</t>
+          <t xml:space="preserve">8a250f761cc363eea77b5980</t>
         </is>
       </c>
       <c r="U20" s="2" t="inlineStr">
@@ -3937,7 +3937,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sample Works 11</t>
+          <t xml:space="preserve">Demo Atelier 10</t>
         </is>
       </c>
       <c r="J21" s="3">
@@ -3990,7 +3990,7 @@
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5e0645b136dbd7f2decaa682</t>
+          <t xml:space="preserve">7943599f6107b8e1f33b116f</t>
         </is>
       </c>
       <c r="U21" s="2" t="inlineStr">
@@ -4132,47 +4132,47 @@
         </is>
       </c>
       <c r="C23" s="3">
-        <v>3548</v>
+        <v>3761</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2013 Wuling Sunshine S</t>
+          <t xml:space="preserve">2022 Toyota GR86</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wuling</t>
+          <t xml:space="preserve">Toyota</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sunshine S</t>
+          <t xml:space="preserve">GR86</t>
         </is>
       </c>
       <c r="G23" s="3">
-        <v>2013</v>
+        <v>2022</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">WUL_HongguangS_20</t>
+          <t xml:space="preserve">TOY_GR86_22</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Paint Lab 07</t>
+          <t xml:space="preserve">Demo ReDownload 90</t>
         </is>
       </c>
       <c r="J23" s="3">
-        <v>14006</v>
+        <v>8478</v>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">デモペイント 022 - ストリート</t>
+          <t xml:space="preserve">デモ再DL完全一致</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">プレビュー版の機能確認用ダミーデータです。テーマ: ストリート。作成者・タイトル・説明・画像・識別情報・FH6表示日付は実データから置き換えています。</t>
+          <t xml:space="preserve">再ダウンロード完全一致の整理機能を確認するためのダミーデータです。</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
@@ -4207,12 +4207,12 @@
       </c>
       <c r="S23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3548_022</t>
+          <t xml:space="preserve">DemoLivery_3761_022</t>
         </is>
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">a2d0ee4f4c78c8c32e907166</t>
+          <t xml:space="preserve">f732dfeca14885528985c557</t>
         </is>
       </c>
       <c r="U23" s="2" t="inlineStr">
@@ -4222,7 +4222,7 @@
       </c>
       <c r="V23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3548_022</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3761_022</t>
         </is>
       </c>
       <c r="W23" s="2" t="inlineStr">
@@ -4274,7 +4274,7 @@
         </is>
       </c>
       <c r="J24" s="3">
-        <v>8627</v>
+        <v>3799</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
@@ -4385,7 +4385,7 @@
         </is>
       </c>
       <c r="J25" s="3">
-        <v>3912</v>
+        <v>8776</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
@@ -4394,7 +4394,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">同一作者・同名候補の比較用ダミーデータ 1 です。画像内容は異なります。</t>
+          <t xml:space="preserve">同一作者・同名候補の比較用ダミーデータ 2 です。画像内容は異なります。</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6c997c4babbafdfc30cc27f1</t>
+          <t xml:space="preserve">201db82e60f24b0fffe33d86</t>
         </is>
       </c>
       <c r="U25" s="2" t="inlineStr">
@@ -4492,11 +4492,11 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preview Garage 06</t>
+          <t xml:space="preserve">Demo Creator 33</t>
         </is>
       </c>
       <c r="J26" s="3">
-        <v>8925</v>
+        <v>4025</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="T26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">e69800671903c61b2fb1e03c</t>
+          <t xml:space="preserve">793c60945cc02c35fd375e04</t>
         </is>
       </c>
       <c r="U26" s="2" t="inlineStr">
@@ -4603,20 +4603,20 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo ReDownload 90</t>
+          <t xml:space="preserve">Preview Similarity 91</t>
         </is>
       </c>
       <c r="J27" s="3">
-        <v>4138</v>
+        <v>9074</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">デモ再DL完全一致</t>
+          <t xml:space="preserve">デモ同一作者・同名</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">再ダウンロード完全一致の整理機能を確認するためのダミーデータです。</t>
+          <t xml:space="preserve">同一作者・同名候補の比較用ダミーデータ 1 です。画像内容は異なります。</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">f732dfeca14885528985c557</t>
+          <t xml:space="preserve">3fc23530096bd7fdc1ecd971</t>
         </is>
       </c>
       <c r="U27" s="2" t="inlineStr">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preview Similarity 91</t>
+          <t xml:space="preserve">Sample Racing 02</t>
         </is>
       </c>
       <c r="J28" s="3">
@@ -4722,12 +4722,12 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">デモ同一作者・同名</t>
+          <t xml:space="preserve">デモペイント 027 - シンプル</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">同一作者・同名候補の比較用ダミーデータ 2 です。画像内容は異なります。</t>
+          <t xml:space="preserve">プレビュー版の機能確認用ダミーデータです。テーマ: シンプル。作成者・タイトル・説明・画像・識別情報・FH6表示日付は実データから置き換えています。</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sample Racing 02</t>
+          <t xml:space="preserve">Preview Studio 03</t>
         </is>
       </c>
       <c r="J34" s="3">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="T34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2241f63f30f18c5b8689f3e9</t>
+          <t xml:space="preserve">530f9843a38c9253a613b2e9</t>
         </is>
       </c>
       <c r="U34" s="2" t="inlineStr">
@@ -5491,7 +5491,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 21</t>
+          <t xml:space="preserve">Preview Studio 03</t>
         </is>
       </c>
       <c r="J35" s="3">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="T35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">b5dd76bfb1fdd9bcc4f2b2d1</t>
+          <t xml:space="preserve">44c44ab5388a265400f672ae</t>
         </is>
       </c>
       <c r="U35" s="2" t="inlineStr">
@@ -5606,7 +5606,7 @@
         </is>
       </c>
       <c r="J36" s="3">
-        <v>5915</v>
+        <v>11755</v>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
@@ -5713,7 +5713,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preview Studio 03</t>
+          <t xml:space="preserve">Demo Creator 34</t>
         </is>
       </c>
       <c r="J37" s="3">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="T37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0774138d6ecf992b03216a8d</t>
+          <t xml:space="preserve">43cd26305d4b60942882ae04</t>
         </is>
       </c>
       <c r="U37" s="2" t="inlineStr">
@@ -5824,11 +5824,11 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preview Studio 03</t>
+          <t xml:space="preserve">Demo Creator 32</t>
         </is>
       </c>
       <c r="J38" s="3">
-        <v>12101</v>
+        <v>6213</v>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
@@ -5877,7 +5877,7 @@
       </c>
       <c r="T38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">641b9564e22f280faa396cda</t>
+          <t xml:space="preserve">794f56182c66c923bc516d2f</t>
         </is>
       </c>
       <c r="U38" s="2" t="inlineStr">
@@ -5935,11 +5935,11 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 34</t>
+          <t xml:space="preserve">DemoWorks 01</t>
         </is>
       </c>
       <c r="J39" s="3">
-        <v>12274</v>
+        <v>1994</v>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
@@ -5988,7 +5988,7 @@
       </c>
       <c r="T39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5304158f666e7f05ea97b623</t>
+          <t xml:space="preserve">198eda3a35c2506fac0b7528</t>
         </is>
       </c>
       <c r="U39" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 31</t>
+          <t xml:space="preserve">Demo Graphics 04</t>
         </is>
       </c>
       <c r="J40" s="3">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="T40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6f6269710cf287a85794565f</t>
+          <t xml:space="preserve">7d26988ab55db23174aa7d3f</t>
         </is>
       </c>
       <c r="U40" s="2" t="inlineStr">
@@ -6130,38 +6130,38 @@
         </is>
       </c>
       <c r="C41" s="3">
-        <v>3761</v>
+        <v>3854</v>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2022 Toyota GR86</t>
+          <t xml:space="preserve">1993 Autozam AZ-1</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toyota</t>
+          <t xml:space="preserve">Autozam</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GR86</t>
+          <t xml:space="preserve">AZ-1</t>
         </is>
       </c>
       <c r="G41" s="3">
-        <v>2022</v>
+        <v>1993</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TOY_GR86_22</t>
+          <t xml:space="preserve">AZM_AZ1_93</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoWorks 01</t>
+          <t xml:space="preserve">Sample Livery 05</t>
         </is>
       </c>
       <c r="J41" s="3">
-        <v>2220</v>
+        <v>6660</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
@@ -6205,12 +6205,12 @@
       </c>
       <c r="S41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3761_040</t>
+          <t xml:space="preserve">DemoLivery_3854_040</t>
         </is>
       </c>
       <c r="T41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">39297cb496c20124f7a5cf38</t>
+          <t xml:space="preserve">309610db78e49d8f58076cf7</t>
         </is>
       </c>
       <c r="U41" s="2" t="inlineStr">
@@ -6220,7 +6220,7 @@
       </c>
       <c r="V41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3761_040</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3854_040</t>
         </is>
       </c>
       <c r="W41" s="2" t="inlineStr">
@@ -6241,34 +6241,34 @@
         </is>
       </c>
       <c r="C42" s="3">
-        <v>3827</v>
+        <v>3865</v>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2023 Hyundai IONIQ 5 N</t>
+          <t xml:space="preserve">1994 Honda Acty</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hyundai</t>
+          <t xml:space="preserve">Honda</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">IONIQ 5 N</t>
+          <t xml:space="preserve">Acty</t>
         </is>
       </c>
       <c r="G42" s="3">
-        <v>2023</v>
+        <v>1994</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HYU_Ioniq5N_23</t>
+          <t xml:space="preserve">HON_Acty_94</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Atelier 10</t>
+          <t xml:space="preserve">Demo Creator 30</t>
         </is>
       </c>
       <c r="J42" s="3">
@@ -6316,12 +6316,12 @@
       </c>
       <c r="S42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3827_041</t>
+          <t xml:space="preserve">DemoLivery_3865_041</t>
         </is>
       </c>
       <c r="T42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">09e21057bf67dd44110d1e20</t>
+          <t xml:space="preserve">ee6de302fcbd4cb797297690</t>
         </is>
       </c>
       <c r="U42" s="2" t="inlineStr">
@@ -6331,7 +6331,7 @@
       </c>
       <c r="V42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3827_041</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3865_041</t>
         </is>
       </c>
       <c r="W42" s="2" t="inlineStr">
@@ -6352,38 +6352,38 @@
         </is>
       </c>
       <c r="C43" s="3">
-        <v>3854</v>
+        <v>3891</v>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1993 Autozam AZ-1</t>
+          <t xml:space="preserve">2024 Lamborghini Revuelto</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Autozam</t>
+          <t xml:space="preserve">Lamborghini</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AZ-1</t>
+          <t xml:space="preserve">Revuelto</t>
         </is>
       </c>
       <c r="G43" s="3">
-        <v>1993</v>
+        <v>2024</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AZM_AZ1_93</t>
+          <t xml:space="preserve">LAM_Revuelto_24</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Graphics 04</t>
+          <t xml:space="preserve">DemoWorks 01</t>
         </is>
       </c>
       <c r="J43" s="3">
-        <v>6958</v>
+        <v>2446</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
@@ -6427,12 +6427,12 @@
       </c>
       <c r="S43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3854_042</t>
+          <t xml:space="preserve">DemoLivery_3891_042</t>
         </is>
       </c>
       <c r="T43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">d87be757bc98d4baddfbe97b</t>
+          <t xml:space="preserve">7db0de3d385085925d37a99c</t>
         </is>
       </c>
       <c r="U43" s="2" t="inlineStr">
@@ -6442,7 +6442,7 @@
       </c>
       <c r="V43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3854_042</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3891_042</t>
         </is>
       </c>
       <c r="W43" s="2" t="inlineStr">
@@ -6463,34 +6463,34 @@
         </is>
       </c>
       <c r="C44" s="3">
-        <v>3865</v>
+        <v>3933</v>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1994 Honda Acty</t>
+          <t xml:space="preserve">1997 Toyota Chaser 2.5 Tourer V</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Honda</t>
+          <t xml:space="preserve">Toyota</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Acty</t>
+          <t xml:space="preserve">Chaser 2.5 Tourer V</t>
         </is>
       </c>
       <c r="G44" s="3">
-        <v>1994</v>
+        <v>1997</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HON_Acty_94</t>
+          <t xml:space="preserve">TOY_Chaser_97</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 30</t>
+          <t xml:space="preserve">DemoWorks 01</t>
         </is>
       </c>
       <c r="J44" s="3">
@@ -6538,12 +6538,12 @@
       </c>
       <c r="S44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3865_043</t>
+          <t xml:space="preserve">DemoLivery_3933_043</t>
         </is>
       </c>
       <c r="T44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">a4273812cc0b4487406c986d</t>
+          <t xml:space="preserve">8377fa23d57b8c1ae668c3f5</t>
         </is>
       </c>
       <c r="U44" s="2" t="inlineStr">
@@ -6553,7 +6553,7 @@
       </c>
       <c r="V44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3865_043</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3933_043</t>
         </is>
       </c>
       <c r="W44" s="2" t="inlineStr">
@@ -6574,38 +6574,38 @@
         </is>
       </c>
       <c r="C45" s="3">
-        <v>3891</v>
+        <v>3953</v>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024 Lamborghini Revuelto</t>
+          <t xml:space="preserve">2023 Porsche 911 Turbo S</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamborghini</t>
+          <t xml:space="preserve">Porsche</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revuelto</t>
+          <t xml:space="preserve">911 Turbo S</t>
         </is>
       </c>
       <c r="G45" s="3">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAM_Revuelto_24</t>
+          <t xml:space="preserve">POR_911TurboS_23</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoWorks 01</t>
+          <t xml:space="preserve">Demo Creator 22</t>
         </is>
       </c>
       <c r="J45" s="3">
-        <v>2672</v>
+        <v>13312</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
@@ -6649,12 +6649,12 @@
       </c>
       <c r="S45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3891_044</t>
+          <t xml:space="preserve">DemoLivery_3953_044</t>
         </is>
       </c>
       <c r="T45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">06073336ae40762ea41922cd</t>
+          <t xml:space="preserve">96c02070a78847b632f55f2d</t>
         </is>
       </c>
       <c r="U45" s="2" t="inlineStr">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="V45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3891_044</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3953_044</t>
         </is>
       </c>
       <c r="W45" s="2" t="inlineStr">
@@ -6685,29 +6685,29 @@
         </is>
       </c>
       <c r="C46" s="3">
-        <v>3933</v>
+        <v>4002</v>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1997 Toyota Chaser 2.5 Tourer V</t>
+          <t xml:space="preserve">2024 Lamborghini Temerario</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toyota</t>
+          <t xml:space="preserve">Lamborghini</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chaser 2.5 Tourer V</t>
+          <t xml:space="preserve">Temerario</t>
         </is>
       </c>
       <c r="G46" s="3">
-        <v>1997</v>
+        <v>2024</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TOY_Chaser_97</t>
+          <t xml:space="preserve">LAM_Temerario_24</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -6760,12 +6760,12 @@
       </c>
       <c r="S46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3933_045</t>
+          <t xml:space="preserve">DemoLivery_4002_045</t>
         </is>
       </c>
       <c r="T46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2df469d119ce38ba872b54f2</t>
+          <t xml:space="preserve">0eb0e33279aae8f73614ab91</t>
         </is>
       </c>
       <c r="U46" s="2" t="inlineStr">
@@ -6775,7 +6775,7 @@
       </c>
       <c r="V46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3933_045</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_4002_045</t>
         </is>
       </c>
       <c r="W46" s="2" t="inlineStr">
@@ -6796,38 +6796,38 @@
         </is>
       </c>
       <c r="C47" s="3">
-        <v>4002</v>
+        <v>4090</v>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024 Lamborghini Temerario</t>
+          <t xml:space="preserve">2001 Mitsubishi Lancer Evolution VI GSR TM Edition</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamborghini</t>
+          <t xml:space="preserve">Mitsubishi</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temerario</t>
+          <t xml:space="preserve">Lancer Evolution VI GSR TM Edition</t>
         </is>
       </c>
       <c r="G47" s="3">
-        <v>2024</v>
+        <v>2001</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAM_Temerario_24</t>
+          <t xml:space="preserve">MIT_LancerEvoVITME_01</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoWorks 01</t>
+          <t xml:space="preserve">Sample Works 11</t>
         </is>
       </c>
       <c r="J47" s="3">
-        <v>7554</v>
+        <v>13658</v>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
@@ -6871,12 +6871,12 @@
       </c>
       <c r="S47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_4002_046</t>
+          <t xml:space="preserve">DemoLivery_4090_046</t>
         </is>
       </c>
       <c r="T47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">42d32c2e3b186f65971a7b70</t>
+          <t xml:space="preserve">196b5836bcf98fdee5675437</t>
         </is>
       </c>
       <c r="U47" s="2" t="inlineStr">
@@ -6886,7 +6886,7 @@
       </c>
       <c r="V47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_4002_046</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_4090_046</t>
         </is>
       </c>
       <c r="W47" s="2" t="inlineStr">
@@ -6907,38 +6907,38 @@
         </is>
       </c>
       <c r="C48" s="3">
-        <v>4090</v>
+        <v>4145</v>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2001 Mitsubishi Lancer Evolution VI GSR TM Edition</t>
+          <t xml:space="preserve">1974 Mazda #123 Mad Mike 808 Wagon 'FURSTY'</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mitsubishi</t>
+          <t xml:space="preserve">Mazda</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lancer Evolution VI GSR TM Edition</t>
+          <t xml:space="preserve">#123 Mad Mike 808 Wagon 'FURSTY'</t>
         </is>
       </c>
       <c r="G48" s="3">
-        <v>2001</v>
+        <v>1974</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MIT_LancerEvoVITME_01</t>
+          <t xml:space="preserve">MAZ_123_808Wagon_74</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preview Factory 12</t>
+          <t xml:space="preserve">Sample Motorsport 08</t>
         </is>
       </c>
       <c r="J48" s="3">
-        <v>13831</v>
+        <v>867</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
@@ -6982,12 +6982,12 @@
       </c>
       <c r="S48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_4090_047</t>
+          <t xml:space="preserve">DemoLivery_4145_047</t>
         </is>
       </c>
       <c r="T48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">b6196de9841adf84edbb3ff7</t>
+          <t xml:space="preserve">03f31d97cd8bab4a283bd9b9</t>
         </is>
       </c>
       <c r="U48" s="2" t="inlineStr">
@@ -6997,7 +6997,7 @@
       </c>
       <c r="V48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_4090_047</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_4145_047</t>
         </is>
       </c>
       <c r="W48" s="2" t="inlineStr">
@@ -7018,38 +7018,38 @@
         </is>
       </c>
       <c r="C49" s="3">
-        <v>4145</v>
+        <v>4163</v>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1974 Mazda #123 Mad Mike 808 Wagon 'FURSTY'</t>
+          <t xml:space="preserve">2013 Wuling Sunshine S Forza Edition</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mazda</t>
+          <t xml:space="preserve">Wuling</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">#123 Mad Mike 808 Wagon 'FURSTY'</t>
+          <t xml:space="preserve">Sunshine S Forza Edition</t>
         </is>
       </c>
       <c r="G49" s="3">
-        <v>1974</v>
+        <v>2013</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAZ_123_808Wagon_74</t>
+          <t xml:space="preserve">WUL_HongguangSFE_20</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sample Motorsport 08</t>
+          <t xml:space="preserve">Demo Creator 21</t>
         </is>
       </c>
       <c r="J49" s="3">
-        <v>88</v>
+        <v>7852</v>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
@@ -7093,12 +7093,12 @@
       </c>
       <c r="S49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_4145_048</t>
+          <t xml:space="preserve">DemoLivery_4163_048</t>
         </is>
       </c>
       <c r="T49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6698fcd1fb9d2e9419cb1b48</t>
+          <t xml:space="preserve">e17351fd70731858d50235db</t>
         </is>
       </c>
       <c r="U49" s="2" t="inlineStr">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="V49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_4145_048</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_4163_048</t>
         </is>
       </c>
       <c r="W49" s="2" t="inlineStr">
@@ -7156,7 +7156,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sample Livery 05</t>
+          <t xml:space="preserve">Preview Garage 06</t>
         </is>
       </c>
       <c r="J50" s="3">
@@ -7209,7 +7209,7 @@
       </c>
       <c r="T50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">21b82484496570b400ff09a0</t>
+          <t xml:space="preserve">bee64e315d30f06ffc1502e0</t>
         </is>
       </c>
       <c r="U50" s="2" t="inlineStr">

</xml_diff>

<commit_message>
:globe_with_meridians: Update public demo for v0.4.60
</commit_message>
<xml_diff>
--- a/fh6-livery-organizer-demo.xlsx
+++ b/fh6-livery-organizer-demo.xlsx
@@ -1801,38 +1801,38 @@
         </is>
       </c>
       <c r="C2" s="3">
-        <v>422</v>
+        <v>296</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2002 Acura RSX Type S</t>
+          <t xml:space="preserve">1998 TVR Cerbera Speed 12</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Acura</t>
+          <t xml:space="preserve">TVR</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RSX Type S</t>
+          <t xml:space="preserve">Cerbera Speed 12</t>
         </is>
       </c>
       <c r="G2" s="3">
-        <v>2002</v>
+        <v>1998</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACU_RSXTypeS_02</t>
+          <t xml:space="preserve">TVR_Cerbera_98</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 19</t>
+          <t xml:space="preserve">Preview Factory 12</t>
         </is>
       </c>
       <c r="J2" s="3">
-        <v>5349</v>
+        <v>10373</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -1876,12 +1876,12 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_0422_001</t>
+          <t xml:space="preserve">DemoLivery_0296_001</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">e779bec68dacd2f7f649e493</t>
+          <t xml:space="preserve">f941263ff6a6f075c61d696f</t>
         </is>
       </c>
       <c r="U2" s="2" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_0422_001</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_0296_001</t>
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr">
@@ -1912,38 +1912,38 @@
         </is>
       </c>
       <c r="C3" s="3">
-        <v>433</v>
+        <v>422</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2005 TVR Sagaris</t>
+          <t xml:space="preserve">2002 Acura RSX Type S</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TVR</t>
+          <t xml:space="preserve">Acura</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sagaris</t>
+          <t xml:space="preserve">RSX Type S</t>
         </is>
       </c>
       <c r="G3" s="3">
-        <v>2005</v>
+        <v>2002</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TVR_Sagaris_05</t>
+          <t xml:space="preserve">ACU_RSXTypeS_02</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 29</t>
+          <t xml:space="preserve">Demo Creator 19</t>
         </is>
       </c>
       <c r="J3" s="3">
-        <v>1426</v>
+        <v>5498</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -1987,12 +1987,12 @@
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_0433_002</t>
+          <t xml:space="preserve">DemoLivery_0422_002</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">d253434b6fa446c3d7c12706</t>
+          <t xml:space="preserve">3923c43da8a23c21d25b6b3f</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_0433_002</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_0422_002</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
@@ -2023,38 +2023,38 @@
         </is>
       </c>
       <c r="C4" s="3">
-        <v>1045</v>
+        <v>615</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1987 Pontiac Firebird Trans Am GTA</t>
+          <t xml:space="preserve">2007 Peugeot 207 Super 2000</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pontiac</t>
+          <t xml:space="preserve">Peugeot</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Firebird Trans Am GTA</t>
+          <t xml:space="preserve">207 Super 2000</t>
         </is>
       </c>
       <c r="G4" s="3">
-        <v>1987</v>
+        <v>2007</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PON_TransAmGTA_87</t>
+          <t xml:space="preserve">PEU_207Super2000_07</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 23</t>
+          <t xml:space="preserve">Demo Creator 22</t>
         </is>
       </c>
       <c r="J4" s="3">
-        <v>293</v>
+        <v>5647</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -2098,12 +2098,12 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_1045_003</t>
+          <t xml:space="preserve">DemoLivery_0615_003</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">efc8f432903d355f23d3e464</t>
+          <t xml:space="preserve">ee84976d6b5c13961a0af0d4</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1045_003</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_0615_003</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
@@ -2134,38 +2134,38 @@
         </is>
       </c>
       <c r="C5" s="3">
-        <v>1124</v>
+        <v>1045</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1980 Abarth Fiat 131</t>
+          <t xml:space="preserve">1987 Pontiac Firebird Trans Am GTA</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abarth</t>
+          <t xml:space="preserve">Pontiac</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fiat 131</t>
+          <t xml:space="preserve">Firebird Trans Am GTA</t>
         </is>
       </c>
       <c r="G5" s="3">
-        <v>1980</v>
+        <v>1987</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FIA_131AbarthStradale_80</t>
+          <t xml:space="preserve">PON_TransAmGTA_87</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 15</t>
+          <t xml:space="preserve">Demo Creator 24</t>
         </is>
       </c>
       <c r="J5" s="3">
-        <v>5796</v>
+        <v>364</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
@@ -2209,12 +2209,12 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_1124_004</t>
+          <t xml:space="preserve">DemoLivery_1045_004</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">e466dd5765184bfee303014d</t>
+          <t xml:space="preserve">c4657a479e4fa929f596865d</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1124_004</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1045_004</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr">
@@ -2245,38 +2245,38 @@
         </is>
       </c>
       <c r="C6" s="3">
-        <v>1130</v>
+        <v>1124</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2011 McLaren 12C Coupé</t>
+          <t xml:space="preserve">1980 Abarth Fiat 131</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">McLaren</t>
+          <t xml:space="preserve">Abarth</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">12C Coupé</t>
+          <t xml:space="preserve">Fiat 131</t>
         </is>
       </c>
       <c r="G6" s="3">
-        <v>2011</v>
+        <v>1980</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCL_MP412C_11</t>
+          <t xml:space="preserve">FIA_131AbarthStradale_80</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 37</t>
+          <t xml:space="preserve">Demo Creator 15</t>
         </is>
       </c>
       <c r="J6" s="3">
-        <v>11065</v>
+        <v>5945</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -2320,12 +2320,12 @@
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_1130_005</t>
+          <t xml:space="preserve">DemoLivery_1124_005</t>
         </is>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">7902fafe68f3da51050fc790</t>
+          <t xml:space="preserve">22a3397f9e872444037c2a64</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1130_005</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1124_005</t>
         </is>
       </c>
       <c r="W6" s="2" t="inlineStr">
@@ -2356,38 +2356,38 @@
         </is>
       </c>
       <c r="C7" s="3">
-        <v>1270</v>
+        <v>1130</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1982 DeLorean DMC-12</t>
+          <t xml:space="preserve">2011 McLaren 12C Coupé</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeLorean</t>
+          <t xml:space="preserve">McLaren</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DMC-12</t>
+          <t xml:space="preserve">12C Coupé</t>
         </is>
       </c>
       <c r="G7" s="3">
-        <v>1982</v>
+        <v>2011</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEL_DMC12_82</t>
+          <t xml:space="preserve">MCL_MP412C_11</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 25</t>
+          <t xml:space="preserve">Demo Creator 38</t>
         </is>
       </c>
       <c r="J7" s="3">
-        <v>6094</v>
+        <v>11238</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
@@ -2431,12 +2431,12 @@
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_1270_006</t>
+          <t xml:space="preserve">DemoLivery_1130_006</t>
         </is>
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">47cb49916fb141df51576857</t>
+          <t xml:space="preserve">a375edb163a1aa37d6eff2b6</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1270_006</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1130_006</t>
         </is>
       </c>
       <c r="W7" s="2" t="inlineStr">
@@ -2467,34 +2467,34 @@
         </is>
       </c>
       <c r="C8" s="3">
-        <v>1382</v>
+        <v>1270</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1990 Subaru LEGACY RS</t>
+          <t xml:space="preserve">1982 DeLorean DMC-12</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Subaru</t>
+          <t xml:space="preserve">DeLorean</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LEGACY RS</t>
+          <t xml:space="preserve">DMC-12</t>
         </is>
       </c>
       <c r="G8" s="3">
-        <v>1990</v>
+        <v>1982</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUB_LegacyRS_90</t>
+          <t xml:space="preserve">DEL_DMC12_82</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 36</t>
+          <t xml:space="preserve">Demo Creator 26</t>
         </is>
       </c>
       <c r="J8" s="3">
@@ -2542,12 +2542,12 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_1382_007</t>
+          <t xml:space="preserve">DemoLivery_1270_007</t>
         </is>
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ae1dc972112209cd988850fd</t>
+          <t xml:space="preserve">1f4a4c92373c72b049d297b6</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1382_007</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1270_007</t>
         </is>
       </c>
       <c r="W8" s="2" t="inlineStr">
@@ -2578,38 +2578,38 @@
         </is>
       </c>
       <c r="C9" s="3">
-        <v>1591</v>
+        <v>1382</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1984 Peugeot 205 Turbo 16</t>
+          <t xml:space="preserve">1990 Subaru LEGACY RS</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peugeot</t>
+          <t xml:space="preserve">Subaru</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">205 Turbo 16</t>
+          <t xml:space="preserve">LEGACY RS</t>
         </is>
       </c>
       <c r="G9" s="3">
-        <v>1984</v>
+        <v>1990</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PEU_205T16_84</t>
+          <t xml:space="preserve">SUB_LegacyRS_90</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 13</t>
+          <t xml:space="preserve">Demo Creator 37</t>
         </is>
       </c>
       <c r="J9" s="3">
-        <v>11584</v>
+        <v>6392</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
@@ -2653,12 +2653,12 @@
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_1591_008</t>
+          <t xml:space="preserve">DemoLivery_1382_008</t>
         </is>
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1435f6e3896f96fffb44b7e0</t>
+          <t xml:space="preserve">e6fa58a842cc5b0ec84f9718</t>
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr">
@@ -2668,7 +2668,7 @@
       </c>
       <c r="V9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1591_008</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1382_008</t>
         </is>
       </c>
       <c r="W9" s="2" t="inlineStr">
@@ -2689,38 +2689,38 @@
         </is>
       </c>
       <c r="C10" s="3">
-        <v>2002</v>
+        <v>1514</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2012 Nissan GT-R Black Edition (R35)</t>
+          <t xml:space="preserve">1973 Mazda RX-3</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nissan</t>
+          <t xml:space="preserve">Mazda</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GT-R Black Edition (R35)</t>
+          <t xml:space="preserve">RX-3</t>
         </is>
       </c>
       <c r="G10" s="3">
-        <v>2012</v>
+        <v>1973</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NIS_GTR_12</t>
+          <t xml:space="preserve">MAZ_RX3_73</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoWorks 01</t>
+          <t xml:space="preserve">Demo Creator 28</t>
         </is>
       </c>
       <c r="J10" s="3">
-        <v>6541</v>
+        <v>2217</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -2764,12 +2764,12 @@
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_2002_009</t>
+          <t xml:space="preserve">DemoLivery_1514_009</t>
         </is>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">7f08e8b73b02a5d5a8dba3b5</t>
+          <t xml:space="preserve">df0173c0c99fffec10a80fcf</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_2002_009</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_1514_009</t>
         </is>
       </c>
       <c r="W10" s="2" t="inlineStr">
@@ -2800,38 +2800,38 @@
         </is>
       </c>
       <c r="C11" s="3">
-        <v>2412</v>
+        <v>2002</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1957 BMW Isetta 300 Export</t>
+          <t xml:space="preserve">2012 Nissan GT-R Black Edition (R35)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">BMW</t>
+          <t xml:space="preserve">Nissan</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Isetta 300 Export</t>
+          <t xml:space="preserve">GT-R Black Edition (R35)</t>
         </is>
       </c>
       <c r="G11" s="3">
-        <v>1957</v>
+        <v>2012</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">bmw_isetta_62</t>
+          <t xml:space="preserve">NIS_GTR_12</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 16</t>
+          <t xml:space="preserve">DemoWorks 01</t>
         </is>
       </c>
       <c r="J11" s="3">
-        <v>790</v>
+        <v>6690</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
@@ -2875,12 +2875,12 @@
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_2412_010</t>
+          <t xml:space="preserve">DemoLivery_2002_010</t>
         </is>
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">295ba194f516f7b88564a168</t>
+          <t xml:space="preserve">6f65a95b424386749d0dfdc1</t>
         </is>
       </c>
       <c r="U11" s="2" t="inlineStr">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_2412_010</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_2002_010</t>
         </is>
       </c>
       <c r="W11" s="2" t="inlineStr">
@@ -2911,38 +2911,38 @@
         </is>
       </c>
       <c r="C12" s="3">
-        <v>2430</v>
+        <v>2412</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2016 Ariel Nomad</t>
+          <t xml:space="preserve">1957 BMW Isetta 300 Export</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ariel</t>
+          <t xml:space="preserve">BMW</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nomad</t>
+          <t xml:space="preserve">Isetta 300 Export</t>
         </is>
       </c>
       <c r="G12" s="3">
-        <v>2016</v>
+        <v>1957</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARI_Nomad_16</t>
+          <t xml:space="preserve">bmw_isetta_62</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 20</t>
+          <t xml:space="preserve">Demo Creator 16</t>
         </is>
       </c>
       <c r="J12" s="3">
-        <v>2443</v>
+        <v>861</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
@@ -2986,12 +2986,12 @@
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_2430_011</t>
+          <t xml:space="preserve">DemoLivery_2412_011</t>
         </is>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">359893763b8db363960bbb34</t>
+          <t xml:space="preserve">20c7e27cc773e7ac269e37a0</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_2430_011</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_2412_011</t>
         </is>
       </c>
       <c r="W12" s="2" t="inlineStr">
@@ -3022,38 +3022,38 @@
         </is>
       </c>
       <c r="C13" s="3">
-        <v>2569</v>
+        <v>2430</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2015 Ultima Evolution Coupe 1020</t>
+          <t xml:space="preserve">2016 Ariel Nomad</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ultima</t>
+          <t xml:space="preserve">Ariel</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolution Coupe 1020</t>
+          <t xml:space="preserve">Nomad</t>
         </is>
       </c>
       <c r="G13" s="3">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ULT_EvolutionCoupe_15</t>
+          <t xml:space="preserve">ARI_Nomad_16</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 27</t>
+          <t xml:space="preserve">Demo Creator 20</t>
         </is>
       </c>
       <c r="J13" s="3">
-        <v>6988</v>
+        <v>2556</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
@@ -3097,12 +3097,12 @@
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_2569_012</t>
+          <t xml:space="preserve">DemoLivery_2430_012</t>
         </is>
       </c>
       <c r="T13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4eb5949ebe53dd6c528e3129</t>
+          <t xml:space="preserve">8b09773eb82c53c3395793dd</t>
         </is>
       </c>
       <c r="U13" s="2" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="V13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_2569_012</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_2430_012</t>
         </is>
       </c>
       <c r="W13" s="2" t="inlineStr">
@@ -3133,38 +3133,38 @@
         </is>
       </c>
       <c r="C14" s="3">
-        <v>2649</v>
+        <v>2569</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2010 Ford Crown Victoria Police Interceptor</t>
+          <t xml:space="preserve">2015 Ultima Evolution Coupe 1020</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ford</t>
+          <t xml:space="preserve">Ultima</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Crown Victoria Police Interceptor</t>
+          <t xml:space="preserve">Evolution Coupe 1020</t>
         </is>
       </c>
       <c r="G14" s="3">
-        <v>2010</v>
+        <v>2015</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">for_crownvictoria_10</t>
+          <t xml:space="preserve">ULT_EvolutionCoupe_15</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 28</t>
+          <t xml:space="preserve">Demo Creator 29</t>
         </is>
       </c>
       <c r="J14" s="3">
-        <v>2669</v>
+        <v>7137</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -3208,12 +3208,12 @@
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_2649_013</t>
+          <t xml:space="preserve">DemoLivery_2569_013</t>
         </is>
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3308a21bc2d460f6c2f91855</t>
+          <t xml:space="preserve">f64918b0fb266ccf114021f1</t>
         </is>
       </c>
       <c r="U14" s="2" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="V14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_2649_013</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_2569_013</t>
         </is>
       </c>
       <c r="W14" s="2" t="inlineStr">
@@ -3244,34 +3244,34 @@
         </is>
       </c>
       <c r="C15" s="3">
-        <v>2987</v>
+        <v>2649</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1962 Peel P50</t>
+          <t xml:space="preserve">2010 Ford Crown Victoria Police Interceptor</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peel</t>
+          <t xml:space="preserve">Ford</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">P50</t>
+          <t xml:space="preserve">Crown Victoria Police Interceptor</t>
         </is>
       </c>
       <c r="G15" s="3">
-        <v>1962</v>
+        <v>2010</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PEE_P50_62</t>
+          <t xml:space="preserve">for_crownvictoria_10</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 31</t>
+          <t xml:space="preserve">Demo Creator 30</t>
         </is>
       </c>
       <c r="J15" s="3">
@@ -3319,12 +3319,12 @@
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_2987_014</t>
+          <t xml:space="preserve">DemoLivery_2649_014</t>
         </is>
       </c>
       <c r="T15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">fbc466f459e9bd8f085b409a</t>
+          <t xml:space="preserve">082acb742ab6816a1f1e21d7</t>
         </is>
       </c>
       <c r="U15" s="2" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="V15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_2987_014</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_2649_014</t>
         </is>
       </c>
       <c r="W15" s="2" t="inlineStr">
@@ -3355,38 +3355,38 @@
         </is>
       </c>
       <c r="C16" s="3">
-        <v>3129</v>
+        <v>2987</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2008 Renault Mégane R26.R</t>
+          <t xml:space="preserve">1962 Peel P50</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Renault</t>
+          <t xml:space="preserve">Peel</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mégane R26.R</t>
+          <t xml:space="preserve">P50</t>
         </is>
       </c>
       <c r="G16" s="3">
-        <v>2008</v>
+        <v>1962</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">REN_MeganeR26R_08</t>
+          <t xml:space="preserve">PEE_P50_62</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoWorks 01</t>
+          <t xml:space="preserve">Demo Creator 32</t>
         </is>
       </c>
       <c r="J16" s="3">
-        <v>7435</v>
+        <v>2895</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
@@ -3430,12 +3430,12 @@
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3129_015</t>
+          <t xml:space="preserve">DemoLivery_2987_015</t>
         </is>
       </c>
       <c r="T16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">97fbe6a47441f3df92652998</t>
+          <t xml:space="preserve">79d61edd7ec092a3f7055201</t>
         </is>
       </c>
       <c r="U16" s="2" t="inlineStr">
@@ -3445,7 +3445,7 @@
       </c>
       <c r="V16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3129_015</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_2987_015</t>
         </is>
       </c>
       <c r="W16" s="2" t="inlineStr">
@@ -3466,34 +3466,34 @@
         </is>
       </c>
       <c r="C17" s="3">
-        <v>3149</v>
+        <v>3129</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2018 Chevrolet Camaro ZL1 1LE</t>
+          <t xml:space="preserve">2008 Renault Mégane R26.R</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chevrolet</t>
+          <t xml:space="preserve">Renault</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Camaro ZL1 1LE</t>
+          <t xml:space="preserve">Mégane R26.R</t>
         </is>
       </c>
       <c r="G17" s="3">
-        <v>2018</v>
+        <v>2008</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CHE_Camaro1LE_18</t>
+          <t xml:space="preserve">REN_MeganeR26R_08</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 26</t>
+          <t xml:space="preserve">DemoWorks 01</t>
         </is>
       </c>
       <c r="J17" s="3">
@@ -3541,12 +3541,12 @@
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3149_016</t>
+          <t xml:space="preserve">DemoLivery_3129_016</t>
         </is>
       </c>
       <c r="T17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">bed25db74411f3081c9f693c</t>
+          <t xml:space="preserve">9d050ba4e5b775e80d0806e8</t>
         </is>
       </c>
       <c r="U17" s="2" t="inlineStr">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="V17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3149_016</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3129_016</t>
         </is>
       </c>
       <c r="W17" s="2" t="inlineStr">
@@ -3577,34 +3577,34 @@
         </is>
       </c>
       <c r="C18" s="3">
-        <v>3211</v>
+        <v>3149</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2017 Aston Martin Vulcan AMR Pro</t>
+          <t xml:space="preserve">2018 Chevrolet Camaro ZL1 1LE</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aston Martin</t>
+          <t xml:space="preserve">Chevrolet</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vulcan AMR Pro</t>
+          <t xml:space="preserve">Camaro ZL1 1LE</t>
         </is>
       </c>
       <c r="G18" s="3">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AST_VulcanAMRPro_19</t>
+          <t xml:space="preserve">CHE_Camaro1LE_18</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 18</t>
+          <t xml:space="preserve">Demo Creator 27</t>
         </is>
       </c>
       <c r="J18" s="3">
@@ -3652,12 +3652,12 @@
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3211_017</t>
+          <t xml:space="preserve">DemoLivery_3149_017</t>
         </is>
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5663cb081a5208f00fc0e669</t>
+          <t xml:space="preserve">b570909be9ecfec70444b32e</t>
         </is>
       </c>
       <c r="U18" s="2" t="inlineStr">
@@ -3667,7 +3667,7 @@
       </c>
       <c r="V18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3211_017</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3149_017</t>
         </is>
       </c>
       <c r="W18" s="2" t="inlineStr">
@@ -3688,34 +3688,34 @@
         </is>
       </c>
       <c r="C19" s="3">
-        <v>3359</v>
+        <v>3211</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2021 Audi RS e-tron GT</t>
+          <t xml:space="preserve">2017 Aston Martin Vulcan AMR Pro</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Audi</t>
+          <t xml:space="preserve">Aston Martin</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RS e-tron GT</t>
+          <t xml:space="preserve">Vulcan AMR Pro</t>
         </is>
       </c>
       <c r="G19" s="3">
-        <v>2021</v>
+        <v>2017</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUD_Etron_18</t>
+          <t xml:space="preserve">AST_VulcanAMRPro_19</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 24</t>
+          <t xml:space="preserve">Demo Creator 18</t>
         </is>
       </c>
       <c r="J19" s="3">
@@ -3763,12 +3763,12 @@
       </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3359_018</t>
+          <t xml:space="preserve">DemoLivery_3211_018</t>
         </is>
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">b64a9dc2626f380ef7bba6b9</t>
+          <t xml:space="preserve">c9c937dae0f8da01e633e5b3</t>
         </is>
       </c>
       <c r="U19" s="2" t="inlineStr">
@@ -3778,7 +3778,7 @@
       </c>
       <c r="V19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3359_018</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3211_018</t>
         </is>
       </c>
       <c r="W19" s="2" t="inlineStr">
@@ -3799,38 +3799,38 @@
         </is>
       </c>
       <c r="C20" s="3">
-        <v>3367</v>
+        <v>3359</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2019 Ferrari F8 Tributo</t>
+          <t xml:space="preserve">2021 Audi RS e-tron GT</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ferrari</t>
+          <t xml:space="preserve">Audi</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">F8 Tributo</t>
+          <t xml:space="preserve">RS e-tron GT</t>
         </is>
       </c>
       <c r="G20" s="3">
-        <v>2019</v>
+        <v>2021</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FER_F8Tributo_20</t>
+          <t xml:space="preserve">AUD_Etron_18</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 17</t>
+          <t xml:space="preserve">Demo Creator 25</t>
         </is>
       </c>
       <c r="J20" s="3">
-        <v>13487</v>
+        <v>8031</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
@@ -3874,12 +3874,12 @@
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3367_019</t>
+          <t xml:space="preserve">DemoLivery_3359_019</t>
         </is>
       </c>
       <c r="T20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8a250f761cc363eea77b5980</t>
+          <t xml:space="preserve">4b52602d7dfb204751414a0e</t>
         </is>
       </c>
       <c r="U20" s="2" t="inlineStr">
@@ -3889,7 +3889,7 @@
       </c>
       <c r="V20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3367_019</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3359_019</t>
         </is>
       </c>
       <c r="W20" s="2" t="inlineStr">
@@ -3910,38 +3910,38 @@
         </is>
       </c>
       <c r="C21" s="3">
-        <v>3494</v>
+        <v>3367</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1968 Alfa Romeo Autodelta Tipo 33/2 Daytona</t>
+          <t xml:space="preserve">2019 Ferrari F8 Tributo</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alfa Romeo</t>
+          <t xml:space="preserve">Ferrari</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Autodelta Tipo 33/2 Daytona</t>
+          <t xml:space="preserve">F8 Tributo</t>
         </is>
       </c>
       <c r="G21" s="3">
-        <v>1968</v>
+        <v>2019</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALF_00_Tipo332_68</t>
+          <t xml:space="preserve">FER_F8Tributo_20</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Atelier 10</t>
+          <t xml:space="preserve">Demo Creator 17</t>
         </is>
       </c>
       <c r="J21" s="3">
-        <v>3460</v>
+        <v>13660</v>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
@@ -3985,12 +3985,12 @@
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3494_020</t>
+          <t xml:space="preserve">DemoLivery_3367_020</t>
         </is>
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">7943599f6107b8e1f33b116f</t>
+          <t xml:space="preserve">bdb410b2f07356fe388a049a</t>
         </is>
       </c>
       <c r="U21" s="2" t="inlineStr">
@@ -4000,7 +4000,7 @@
       </c>
       <c r="V21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3494_020</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3367_020</t>
         </is>
       </c>
       <c r="W21" s="2" t="inlineStr">
@@ -4021,38 +4021,38 @@
         </is>
       </c>
       <c r="C22" s="3">
-        <v>3523</v>
+        <v>3494</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2020 Formula Drift #151 Toyota GR Supra</t>
+          <t xml:space="preserve">1968 Alfa Romeo Autodelta Tipo 33/2 Daytona</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Formula Drift</t>
+          <t xml:space="preserve">Alfa Romeo</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">#151 Toyota GR Supra</t>
+          <t xml:space="preserve">Autodelta Tipo 33/2 Daytona</t>
         </is>
       </c>
       <c r="G22" s="3">
-        <v>2020</v>
+        <v>1968</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TOY_151_SupraGRFD_20</t>
+          <t xml:space="preserve">ALF_00_Tipo332_68</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 35</t>
+          <t xml:space="preserve">Preview Design 09</t>
         </is>
       </c>
       <c r="J22" s="3">
-        <v>8329</v>
+        <v>3573</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
@@ -4096,12 +4096,12 @@
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3523_021</t>
+          <t xml:space="preserve">DemoLivery_3494_021</t>
         </is>
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1abc974271e45faebc729373</t>
+          <t xml:space="preserve">d2ce08f8e04a1c5f828a22bd</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
@@ -4111,7 +4111,7 @@
       </c>
       <c r="V22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3523_021</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3494_021</t>
         </is>
       </c>
       <c r="W22" s="2" t="inlineStr">
@@ -4132,34 +4132,34 @@
         </is>
       </c>
       <c r="C23" s="3">
-        <v>3761</v>
+        <v>3523</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2022 Toyota GR86</t>
+          <t xml:space="preserve">2020 Formula Drift #151 Toyota GR Supra</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toyota</t>
+          <t xml:space="preserve">Formula Drift</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GR86</t>
+          <t xml:space="preserve">#151 Toyota GR Supra</t>
         </is>
       </c>
       <c r="G23" s="3">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TOY_GR86_22</t>
+          <t xml:space="preserve">TOY_151_SupraGRFD_20</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo ReDownload 90</t>
+          <t xml:space="preserve">Demo Creator 36</t>
         </is>
       </c>
       <c r="J23" s="3">
@@ -4167,12 +4167,12 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">デモ再DL完全一致</t>
+          <t xml:space="preserve">デモペイント 022 - ストリート</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">再ダウンロード完全一致の整理機能を確認するためのダミーデータです。</t>
+          <t xml:space="preserve">プレビュー版の機能確認用ダミーデータです。テーマ: ストリート。作成者・タイトル・説明・画像・識別情報・FH6表示日付は実データから置き換えています。</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
@@ -4207,12 +4207,12 @@
       </c>
       <c r="S23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3761_022</t>
+          <t xml:space="preserve">DemoLivery_3523_022</t>
         </is>
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">f732dfeca14885528985c557</t>
+          <t xml:space="preserve">40f3dd38c99e7d90c18132c7</t>
         </is>
       </c>
       <c r="U23" s="2" t="inlineStr">
@@ -4222,7 +4222,7 @@
       </c>
       <c r="V23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3761_022</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3523_022</t>
         </is>
       </c>
       <c r="W23" s="2" t="inlineStr">
@@ -4274,7 +4274,7 @@
         </is>
       </c>
       <c r="J24" s="3">
-        <v>3799</v>
+        <v>8627</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
@@ -4385,7 +4385,7 @@
         </is>
       </c>
       <c r="J25" s="3">
-        <v>8776</v>
+        <v>3912</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
@@ -4394,7 +4394,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">同一作者・同名候補の比較用ダミーデータ 2 です。画像内容は異なります。</t>
+          <t xml:space="preserve">同一作者・同名候補の比較用ダミーデータ 1 です。画像内容は異なります。</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">201db82e60f24b0fffe33d86</t>
+          <t xml:space="preserve">5cb8fa1398ec9a8fc4b171d8</t>
         </is>
       </c>
       <c r="U25" s="2" t="inlineStr">
@@ -4492,11 +4492,11 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 33</t>
+          <t xml:space="preserve">Demo Paint Lab 07</t>
         </is>
       </c>
       <c r="J26" s="3">
-        <v>4025</v>
+        <v>8925</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="T26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">793c60945cc02c35fd375e04</t>
+          <t xml:space="preserve">7729fe34381e5b47f3cb5c97</t>
         </is>
       </c>
       <c r="U26" s="2" t="inlineStr">
@@ -4603,20 +4603,20 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preview Similarity 91</t>
+          <t xml:space="preserve">Demo ReDownload 90</t>
         </is>
       </c>
       <c r="J27" s="3">
-        <v>9074</v>
+        <v>4138</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">デモ同一作者・同名</t>
+          <t xml:space="preserve">デモ再DL完全一致</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">同一作者・同名候補の比較用ダミーデータ 1 です。画像内容は異なります。</t>
+          <t xml:space="preserve">再ダウンロード完全一致の整理機能を確認するためのダミーデータです。</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3fc23530096bd7fdc1ecd971</t>
+          <t xml:space="preserve">f732dfeca14885528985c557</t>
         </is>
       </c>
       <c r="U27" s="2" t="inlineStr">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sample Racing 02</t>
+          <t xml:space="preserve">Preview Similarity 91</t>
         </is>
       </c>
       <c r="J28" s="3">
@@ -4722,12 +4722,12 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">デモペイント 027 - シンプル</t>
+          <t xml:space="preserve">デモ同一作者・同名</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">プレビュー版の機能確認用ダミーデータです。テーマ: シンプル。作成者・タイトル・説明・画像・識別情報・FH6表示日付は実データから置き換えています。</t>
+          <t xml:space="preserve">同一作者・同名候補の比較用ダミーデータ 2 です。画像内容は異なります。</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preview Studio 03</t>
+          <t xml:space="preserve">Sample Racing 02</t>
         </is>
       </c>
       <c r="J34" s="3">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="T34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">530f9843a38c9253a613b2e9</t>
+          <t xml:space="preserve">2241f63f30f18c5b8689f3e9</t>
         </is>
       </c>
       <c r="U34" s="2" t="inlineStr">
@@ -5713,7 +5713,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 34</t>
+          <t xml:space="preserve">Demo Creator 35</t>
         </is>
       </c>
       <c r="J37" s="3">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="T37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">43cd26305d4b60942882ae04</t>
+          <t xml:space="preserve">a130bccd508c346f8a75330e</t>
         </is>
       </c>
       <c r="U37" s="2" t="inlineStr">
@@ -5824,7 +5824,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 32</t>
+          <t xml:space="preserve">Demo Creator 33</t>
         </is>
       </c>
       <c r="J38" s="3">
@@ -5877,7 +5877,7 @@
       </c>
       <c r="T38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">794f56182c66c923bc516d2f</t>
+          <t xml:space="preserve">407c464683b6f4f495ff5e2d</t>
         </is>
       </c>
       <c r="U38" s="2" t="inlineStr">
@@ -6130,38 +6130,38 @@
         </is>
       </c>
       <c r="C41" s="3">
-        <v>3854</v>
+        <v>3761</v>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1993 Autozam AZ-1</t>
+          <t xml:space="preserve">2022 Toyota GR86</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Autozam</t>
+          <t xml:space="preserve">Toyota</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AZ-1</t>
+          <t xml:space="preserve">GR86</t>
         </is>
       </c>
       <c r="G41" s="3">
-        <v>1993</v>
+        <v>2022</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AZM_AZ1_93</t>
+          <t xml:space="preserve">TOY_GR86_22</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sample Livery 05</t>
+          <t xml:space="preserve">Demo Creator 13</t>
         </is>
       </c>
       <c r="J41" s="3">
-        <v>6660</v>
+        <v>12620</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
@@ -6205,12 +6205,12 @@
       </c>
       <c r="S41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3854_040</t>
+          <t xml:space="preserve">DemoLivery_3761_040</t>
         </is>
       </c>
       <c r="T41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">309610db78e49d8f58076cf7</t>
+          <t xml:space="preserve">578d6401f06b2e8ee50a6ab6</t>
         </is>
       </c>
       <c r="U41" s="2" t="inlineStr">
@@ -6220,7 +6220,7 @@
       </c>
       <c r="V41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3854_040</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3761_040</t>
         </is>
       </c>
       <c r="W41" s="2" t="inlineStr">
@@ -6241,34 +6241,34 @@
         </is>
       </c>
       <c r="C42" s="3">
-        <v>3865</v>
+        <v>3854</v>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1994 Honda Acty</t>
+          <t xml:space="preserve">1993 Autozam AZ-1</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Honda</t>
+          <t xml:space="preserve">Autozam</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Acty</t>
+          <t xml:space="preserve">AZ-1</t>
         </is>
       </c>
       <c r="G42" s="3">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HON_Acty_94</t>
+          <t xml:space="preserve">AZM_AZ1_93</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 30</t>
+          <t xml:space="preserve">Sample Livery 05</t>
         </is>
       </c>
       <c r="J42" s="3">
@@ -6316,12 +6316,12 @@
       </c>
       <c r="S42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3865_041</t>
+          <t xml:space="preserve">DemoLivery_3854_041</t>
         </is>
       </c>
       <c r="T42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ee6de302fcbd4cb797297690</t>
+          <t xml:space="preserve">cd805d6b69f6edd6b0eac2ec</t>
         </is>
       </c>
       <c r="U42" s="2" t="inlineStr">
@@ -6331,7 +6331,7 @@
       </c>
       <c r="V42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3865_041</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3854_041</t>
         </is>
       </c>
       <c r="W42" s="2" t="inlineStr">
@@ -6352,38 +6352,38 @@
         </is>
       </c>
       <c r="C43" s="3">
-        <v>3891</v>
+        <v>3865</v>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024 Lamborghini Revuelto</t>
+          <t xml:space="preserve">1994 Honda Acty</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamborghini</t>
+          <t xml:space="preserve">Honda</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revuelto</t>
+          <t xml:space="preserve">Acty</t>
         </is>
       </c>
       <c r="G43" s="3">
-        <v>2024</v>
+        <v>1994</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAM_Revuelto_24</t>
+          <t xml:space="preserve">HON_Acty_94</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoWorks 01</t>
+          <t xml:space="preserve">Demo Creator 31</t>
         </is>
       </c>
       <c r="J43" s="3">
-        <v>2446</v>
+        <v>6958</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
@@ -6427,12 +6427,12 @@
       </c>
       <c r="S43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3891_042</t>
+          <t xml:space="preserve">DemoLivery_3865_042</t>
         </is>
       </c>
       <c r="T43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">7db0de3d385085925d37a99c</t>
+          <t xml:space="preserve">6d055e7b8b6781831c08f4b4</t>
         </is>
       </c>
       <c r="U43" s="2" t="inlineStr">
@@ -6442,7 +6442,7 @@
       </c>
       <c r="V43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3891_042</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3865_042</t>
         </is>
       </c>
       <c r="W43" s="2" t="inlineStr">
@@ -6463,29 +6463,29 @@
         </is>
       </c>
       <c r="C44" s="3">
-        <v>3933</v>
+        <v>3891</v>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1997 Toyota Chaser 2.5 Tourer V</t>
+          <t xml:space="preserve">2024 Lamborghini Revuelto</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toyota</t>
+          <t xml:space="preserve">Lamborghini</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chaser 2.5 Tourer V</t>
+          <t xml:space="preserve">Revuelto</t>
         </is>
       </c>
       <c r="G44" s="3">
-        <v>1997</v>
+        <v>2024</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TOY_Chaser_97</t>
+          <t xml:space="preserve">LAM_Revuelto_24</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -6494,7 +6494,7 @@
         </is>
       </c>
       <c r="J44" s="3">
-        <v>7107</v>
+        <v>2559</v>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
@@ -6538,12 +6538,12 @@
       </c>
       <c r="S44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3933_043</t>
+          <t xml:space="preserve">DemoLivery_3891_043</t>
         </is>
       </c>
       <c r="T44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8377fa23d57b8c1ae668c3f5</t>
+          <t xml:space="preserve">e02692c1360826db52caeedc</t>
         </is>
       </c>
       <c r="U44" s="2" t="inlineStr">
@@ -6553,7 +6553,7 @@
       </c>
       <c r="V44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3933_043</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3891_043</t>
         </is>
       </c>
       <c r="W44" s="2" t="inlineStr">
@@ -6574,38 +6574,38 @@
         </is>
       </c>
       <c r="C45" s="3">
-        <v>3953</v>
+        <v>3933</v>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2023 Porsche 911 Turbo S</t>
+          <t xml:space="preserve">1997 Toyota Chaser 2.5 Tourer V</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Porsche</t>
+          <t xml:space="preserve">Toyota</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">911 Turbo S</t>
+          <t xml:space="preserve">Chaser 2.5 Tourer V</t>
         </is>
       </c>
       <c r="G45" s="3">
-        <v>2023</v>
+        <v>1997</v>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">POR_911TurboS_23</t>
+          <t xml:space="preserve">TOY_Chaser_97</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo Creator 22</t>
+          <t xml:space="preserve">DemoWorks 01</t>
         </is>
       </c>
       <c r="J45" s="3">
-        <v>13312</v>
+        <v>7256</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
@@ -6649,12 +6649,12 @@
       </c>
       <c r="S45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_3953_044</t>
+          <t xml:space="preserve">DemoLivery_3933_044</t>
         </is>
       </c>
       <c r="T45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">96c02070a78847b632f55f2d</t>
+          <t xml:space="preserve">a324b8c97f13f3bc61434dea</t>
         </is>
       </c>
       <c r="U45" s="2" t="inlineStr">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="V45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3953_044</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3933_044</t>
         </is>
       </c>
       <c r="W45" s="2" t="inlineStr">
@@ -6685,38 +6685,38 @@
         </is>
       </c>
       <c r="C46" s="3">
-        <v>4002</v>
+        <v>3953</v>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024 Lamborghini Temerario</t>
+          <t xml:space="preserve">2023 Porsche 911 Turbo S</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamborghini</t>
+          <t xml:space="preserve">Porsche</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temerario</t>
+          <t xml:space="preserve">911 Turbo S</t>
         </is>
       </c>
       <c r="G46" s="3">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAM_Temerario_24</t>
+          <t xml:space="preserve">POR_911TurboS_23</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoWorks 01</t>
+          <t xml:space="preserve">Demo Creator 23</t>
         </is>
       </c>
       <c r="J46" s="3">
-        <v>7405</v>
+        <v>13485</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
@@ -6760,12 +6760,12 @@
       </c>
       <c r="S46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_4002_045</t>
+          <t xml:space="preserve">DemoLivery_3953_045</t>
         </is>
       </c>
       <c r="T46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0eb0e33279aae8f73614ab91</t>
+          <t xml:space="preserve">dcdcffb258cdfb45997314f8</t>
         </is>
       </c>
       <c r="U46" s="2" t="inlineStr">
@@ -6775,7 +6775,7 @@
       </c>
       <c r="V46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_4002_045</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_3953_045</t>
         </is>
       </c>
       <c r="W46" s="2" t="inlineStr">
@@ -6796,38 +6796,38 @@
         </is>
       </c>
       <c r="C47" s="3">
-        <v>4090</v>
+        <v>4002</v>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2001 Mitsubishi Lancer Evolution VI GSR TM Edition</t>
+          <t xml:space="preserve">2024 Lamborghini Temerario</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mitsubishi</t>
+          <t xml:space="preserve">Lamborghini</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lancer Evolution VI GSR TM Edition</t>
+          <t xml:space="preserve">Temerario</t>
         </is>
       </c>
       <c r="G47" s="3">
-        <v>2001</v>
+        <v>2024</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MIT_LancerEvoVITME_01</t>
+          <t xml:space="preserve">LAM_Temerario_24</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sample Works 11</t>
+          <t xml:space="preserve">DemoWorks 01</t>
         </is>
       </c>
       <c r="J47" s="3">
-        <v>13658</v>
+        <v>7554</v>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
@@ -6871,12 +6871,12 @@
       </c>
       <c r="S47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_4090_046</t>
+          <t xml:space="preserve">DemoLivery_4002_046</t>
         </is>
       </c>
       <c r="T47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">196b5836bcf98fdee5675437</t>
+          <t xml:space="preserve">42d32c2e3b186f65971a7b70</t>
         </is>
       </c>
       <c r="U47" s="2" t="inlineStr">
@@ -6886,7 +6886,7 @@
       </c>
       <c r="V47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_4090_046</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_4002_046</t>
         </is>
       </c>
       <c r="W47" s="2" t="inlineStr">
@@ -6907,38 +6907,38 @@
         </is>
       </c>
       <c r="C48" s="3">
-        <v>4145</v>
+        <v>4090</v>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1974 Mazda #123 Mad Mike 808 Wagon 'FURSTY'</t>
+          <t xml:space="preserve">2001 Mitsubishi Lancer Evolution VI GSR TM Edition</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mazda</t>
+          <t xml:space="preserve">Mitsubishi</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">#123 Mad Mike 808 Wagon 'FURSTY'</t>
+          <t xml:space="preserve">Lancer Evolution VI GSR TM Edition</t>
         </is>
       </c>
       <c r="G48" s="3">
-        <v>1974</v>
+        <v>2001</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAZ_123_808Wagon_74</t>
+          <t xml:space="preserve">MIT_LancerEvoVITME_01</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sample Motorsport 08</t>
+          <t xml:space="preserve">Demo Atelier 10</t>
         </is>
       </c>
       <c r="J48" s="3">
-        <v>867</v>
+        <v>13831</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
@@ -6982,12 +6982,12 @@
       </c>
       <c r="S48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DemoLivery_4145_047</t>
+          <t xml:space="preserve">DemoLivery_4090_047</t>
         </is>
       </c>
       <c r="T48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">03f31d97cd8bab4a283bd9b9</t>
+          <t xml:space="preserve">8846411f0c7e6c426407734c</t>
         </is>
       </c>
       <c r="U48" s="2" t="inlineStr">
@@ -6997,7 +6997,7 @@
       </c>
       <c r="V48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_4145_047</t>
+          <t xml:space="preserve">C:\Demo\FH6\GameSave\pgs\DemoProfile\ContainersRoot\DemoLivery_4090_047</t>
         </is>
       </c>
       <c r="W48" s="2" t="inlineStr">
@@ -7267,7 +7267,7 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Preview Design 09</t>
+          <t xml:space="preserve">Sample Motorsport 08</t>
         </is>
       </c>
       <c r="J51" s="3">
@@ -7320,7 +7320,7 @@
       </c>
       <c r="T51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3ba453248dafc3271221e4e6</t>
+          <t xml:space="preserve">4a167324b145be97170a1974</t>
         </is>
       </c>
       <c r="U51" s="2" t="inlineStr">

</xml_diff>